<commit_message>
Regenerate 2030 _latest bundles + figure_data from full release run
Outputs of `sbatch scripts/sbatch_release.sh` (vintage 202605261319) after
the BLSMM figure cleanup port: ai_fiscal_2030_latest.xlsx and the
publishable equivalent now carry the refreshed `blsmm_debt_to_gdp` sheet,
and figure_data_2030.xlsx is regenerated from the same release run so the
data backing the figure suite stays in sync.
</commit_message>
<xml_diff>
--- a/results/aggregates/ai_fiscal_2030_latest.xlsx
+++ b/results/aggregates/ai_fiscal_2030_latest.xlsx
@@ -37,7 +37,7 @@
     <t xml:space="preserve">Generated</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-05-26 12:18:03 EDT</t>
+    <t xml:space="preserve">2026-05-26 13:27:04 EDT</t>
   </si>
   <si>
     <t xml:space="preserve">Policy year</t>
@@ -49,13 +49,13 @@
     <t xml:space="preserve">Tax-Simulator vintage</t>
   </si>
   <si>
-    <t xml:space="preserve">202605261209</t>
+    <t xml:space="preserve">202605261319</t>
   </si>
   <si>
     <t xml:space="preserve">Tax-Simulator output root</t>
   </si>
   <si>
-    <t xml:space="preserve">/nfs/roberts/project/pi_nrs36/ji252/scratch/tax_sim/model_data/Tax-Simulator/v1/202605261209</t>
+    <t xml:space="preserve">/nfs/roberts/project/pi_nrs36/ji252/scratch/tax_sim/model_data/Tax-Simulator/v1/202605261319</t>
   </si>
   <si>
     <t xml:space="preserve">Runscript</t>
@@ -85,7 +85,7 @@
     <t xml:space="preserve">ai_fiscal git rev</t>
   </si>
   <si>
-    <t xml:space="preserve">41bbc6df3e2b</t>
+    <t xml:space="preserve">471d9124dd00</t>
   </si>
   <si>
     <t xml:space="preserve">Orchestrator argv</t>

</xml_diff>

<commit_message>
results: regenerate 2030 deliverables (full-grid run, vintage 202606221535)
Full 18-cell x 3-flavor release run (orchestrator exit 0): refreshes the
two tracked _latest.xlsx bundles (with the BLSMM debt/GDP sheet) and the
70-PNG figure suite + figure_data workbook for policy year 2030.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/aggregates/ai_fiscal_2030_latest.xlsx
+++ b/results/aggregates/ai_fiscal_2030_latest.xlsx
@@ -37,7 +37,7 @@
     <t xml:space="preserve">Generated</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-05-26 13:27:04 EDT</t>
+    <t xml:space="preserve">2026-06-22 15:41:47 EDT</t>
   </si>
   <si>
     <t xml:space="preserve">Policy year</t>
@@ -49,19 +49,19 @@
     <t xml:space="preserve">Tax-Simulator vintage</t>
   </si>
   <si>
-    <t xml:space="preserve">202605261319</t>
+    <t xml:space="preserve">202606221535</t>
   </si>
   <si>
     <t xml:space="preserve">Tax-Simulator output root</t>
   </si>
   <si>
-    <t xml:space="preserve">/nfs/roberts/project/pi_nrs36/ji252/scratch/tax_sim/model_data/Tax-Simulator/v1/202605261319</t>
+    <t xml:space="preserve">/nfs/roberts/scratch/pi_nrs36/jar335/model_data/Tax-Simulator/v1/202606221535</t>
   </si>
   <si>
     <t xml:space="preserve">Runscript</t>
   </si>
   <si>
-    <t xml:space="preserve">/nfs/roberts/project/pi_nrs36/ji252/Repositories/Tax-Simulator/config/runscripts/private/ai_fiscal.csv</t>
+    <t xml:space="preserve">/nfs/roberts/project/pi_nrs36/ji252/repos/Tax-Simulator/config/runscripts/private/ai_fiscal.csv</t>
   </si>
   <si>
     <t xml:space="preserve">Scenarios</t>
@@ -82,10 +82,10 @@
     <t xml:space="preserve">R version 4.4.2 (2024-10-31)</t>
   </si>
   <si>
-    <t xml:space="preserve">ai_fiscal git rev</t>
-  </si>
-  <si>
-    <t xml:space="preserve">471d9124dd00</t>
+    <t xml:space="preserve">AI-Fiscal git rev</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f832339471cb</t>
   </si>
   <si>
     <t xml:space="preserve">Orchestrator argv</t>
@@ -676,7 +676,7 @@
     <t xml:space="preserve">CBO_CIT$ = cit_to_gdp_baseline_year * gdp_baseline_year_B$</t>
   </si>
   <si>
-    <t xml:space="preserve">0.013 * 37,391 = $486.1B (2030)</t>
+    <t xml:space="preserve">cit_to_gdp_baseline_year * gdp_baseline_year_B$ (from scenario_params.yaml)</t>
   </si>
   <si>
     <t xml:space="preserve">CBO 2025 Budget and Economic Outlook (publication 62105), Table 1, 2030 federal CIT / GDP, applied to 2030 nominal GDP.</t>
@@ -22762,7 +22762,7 @@
   <cols>
     <col min="1" max="1" width="38.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="72.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="31.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="75.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="60.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="60.71" hidden="0" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
results: regenerate 2030 deliverables under aligned notation (vintage 202606300013)
Re-run of the full grid on the notation-aligned code. Workbook label
sheets (parameters_per_variant, labor_inequality, scenario_guide) now
print theta1_k/g_y/g_k/g_l in place of s1/gy/gk/alpha; results sheets
(revenue/income/gini/share/decomp) are unchanged -- the rename moved no
numbers. Run metadata updated to the ji252 vintage.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/aggregates/ai_fiscal_2030_latest.xlsx
+++ b/results/aggregates/ai_fiscal_2030_latest.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="444">
   <si>
     <t xml:space="preserve">field</t>
   </si>
@@ -37,7 +37,7 @@
     <t xml:space="preserve">Generated</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-06-22 15:41:47 EDT</t>
+    <t xml:space="preserve">2026-06-30 00:20:45 EDT</t>
   </si>
   <si>
     <t xml:space="preserve">Policy year</t>
@@ -49,13 +49,13 @@
     <t xml:space="preserve">Tax-Simulator vintage</t>
   </si>
   <si>
-    <t xml:space="preserve">202606221535</t>
+    <t xml:space="preserve">202606300013</t>
   </si>
   <si>
     <t xml:space="preserve">Tax-Simulator output root</t>
   </si>
   <si>
-    <t xml:space="preserve">/nfs/roberts/scratch/pi_nrs36/jar335/model_data/Tax-Simulator/v1/202606221535</t>
+    <t xml:space="preserve">/nfs/roberts/scratch/pi_nrs36/ji252/model_data/Tax-Simulator/v1/202606300013</t>
   </si>
   <si>
     <t xml:space="preserve">Runscript</t>
@@ -85,7 +85,7 @@
     <t xml:space="preserve">AI-Fiscal git rev</t>
   </si>
   <si>
-    <t xml:space="preserve">f832339471cb</t>
+    <t xml:space="preserve">4a1111ae1e12</t>
   </si>
   <si>
     <t xml:space="preserve">Orchestrator argv</t>
@@ -127,10 +127,10 @@
     <t xml:space="preserve">5-yr cumulative shock target</t>
   </si>
   <si>
-    <t xml:space="preserve">K1 = s1*(1+gy); L1 = (1-s1)*(1+gy); gk = (K1-K0)/K0; alpha = (1/gk) * (L1-L0)/L0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s1=0.450, gy=0.0060 -&gt; gk ≈ +1.7%,  alpha ≈ -0.18 -&gt; labor -0.3%  (Slow)</t>
+    <t xml:space="preserve">g_k = (theta1_k*(1+g_y) - theta0_k)/theta0_k; g_l = (theta1_l*(1+g_y) - theta0_l)/theta0_l</t>
+  </si>
+  <si>
+    <t xml:space="preserve">theta1_k=0.450, g_y=0.0060 -&gt; g_k ≈ +1.7%,  g_l ≈ -0.3%  (Slow)</t>
   </si>
   <si>
     <t xml:space="preserve">Mildest variant. Karger 2026 NBER w35046: Table 39 (labor share) and Table 19 (median 2030 annualized GDP growth under AI), Total column, median.</t>
@@ -145,7 +145,7 @@
     <t xml:space="preserve">(same as S)</t>
   </si>
   <si>
-    <t xml:space="preserve">s1=0.462, gy=0.0358 -&gt; gk ≈ +7.5%,  alpha ≈ +0.05 -&gt; labor +0.4%  (Moderate)</t>
+    <t xml:space="preserve">theta1_k=0.462, g_y=0.0358 -&gt; g_k ≈ +7.5%,  g_l ≈ +0.4%  (Moderate)</t>
   </si>
   <si>
     <t xml:space="preserve">Karger Tables 39 / 19.</t>
@@ -157,7 +157,7 @@
     <t xml:space="preserve">Rapid</t>
   </si>
   <si>
-    <t xml:space="preserve">s1=0.487, gy=0.0716 -&gt; gk ≈ +17.3%, alpha ≈ -0.05 -&gt; labor -0.9% (Rapid)</t>
+    <t xml:space="preserve">theta1_k=0.487, g_y=0.0716 -&gt; g_k ≈ +17.3%, g_l ≈ -0.9% (Rapid)</t>
   </si>
   <si>
     <t xml:space="preserve">Most capital-biased. Karger Tables 39 / 19.</t>
@@ -169,10 +169,10 @@
     <t xml:space="preserve">Reallocate</t>
   </si>
   <si>
-    <t xml:space="preserve">Karger labor-share decline: s1 from yaml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s1 from yaml shock.variants.&lt;variant&gt;.s1; gk and alpha derived as above.</t>
+    <t xml:space="preserve">Karger labor-share decline: theta1_k from yaml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">theta1_k from yaml shock.variants.&lt;variant&gt;.theta1_k; g_k and g_l derived as above.</t>
   </si>
   <si>
     <t xml:space="preserve">Canonical AI-growth-plus-reallocation shock.</t>
@@ -187,13 +187,13 @@
     <t xml:space="preserve">Fixed share</t>
   </si>
   <si>
-    <t xml:space="preserve">Hold labor-capital share at baseline: s1 := 1 - L0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s1 = 1 - L0 = K0  =&gt;  gk = gy, alpha = 1; labor and capital both grow at gy.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paired twin of R: same gy, labor and capital both scale by (1+gy).</t>
+    <t xml:space="preserve">Hold labor-capital share at baseline: theta1_k := theta0_k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">theta1_k = theta0_k  =&gt;  g_k = g_l = g_y; labor and capital both grow at g_y.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paired twin of R: same g_y, labor and capital both scale by (1+g_y).</t>
   </si>
   <si>
     <t xml:space="preserve">Fixed-share mode: the labor-capital split is preserved. Isolates the AI growth channel from the reallocation channel.</t>
@@ -208,13 +208,13 @@
     <t xml:space="preserve">Compressive</t>
   </si>
   <si>
-    <t xml:space="preserve">Log-affine, sigma_S2 = 1 - k_inequality * gy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ln(YiL1) = mu1 + sigma_S2 * (ln(YiL0) - mu0); sigma_S2 = 1 - k_inequality * gy; mu1 via uniroot to hit L1$</t>
-  </si>
-  <si>
-    <t xml:space="preserve">k_inequality = 1 by default (config: labor_inequality.k). See labor_inequality sheet for per-variant sigma_S2.</t>
+    <t xml:space="preserve">Log-affine, lambda_S2 = 1 - k_inequality * g_y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ln(y_l1) = mu1 + lambda_S2 * (ln(y_l) - mu0); lambda_S2 = 1 - k_inequality * g_y; mu1 via uniroot to hit Y1^L$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">k_inequality = 1 by default (config: labor_inequality.k). See labor_inequality sheet for per-variant lambda_S2.</t>
   </si>
   <si>
     <t xml:space="preserve">Reduces labor-income inequality. Rationale: AI commoditizes high-skill premia (top wages pulled toward mean).</t>
@@ -229,7 +229,7 @@
     <t xml:space="preserve">Uniform scaling</t>
   </si>
   <si>
-    <t xml:space="preserve">YiL1 = rho * YiL0, rho = L1$ / L0$</t>
+    <t xml:space="preserve">y_l1 = rho * y_l, rho = Y1^L$ / Y0^L$</t>
   </si>
   <si>
     <t xml:space="preserve">—</t>
@@ -244,13 +244,13 @@
     <t xml:space="preserve">Expansive</t>
   </si>
   <si>
-    <t xml:space="preserve">Log-affine, sigma_S3 = 1 + k_inequality * gy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ln(YiL1) = mu1 + sigma_S3 * (ln(YiL0) - mu0); sigma_S3 = 1 + k_inequality * gy; mu1 via uniroot to hit L1$</t>
-  </si>
-  <si>
-    <t xml:space="preserve">k_inequality = 1 by default (config: labor_inequality.k). See labor_inequality sheet for per-variant sigma_S3.</t>
+    <t xml:space="preserve">Log-affine, lambda_S3 = 1 + k_inequality * g_y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ln(y_l1) = mu1 + lambda_S3 * (ln(y_l) - mu0); lambda_S3 = 1 + k_inequality * g_y; mu1 via uniroot to hit Y1^L$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">k_inequality = 1 by default (config: labor_inequality.k). See labor_inequality sheet for per-variant lambda_S3.</t>
   </si>
   <si>
     <t xml:space="preserve">Increases labor-income inequality. Rationale: AI super-charges top earners (winner-take-most).</t>
@@ -271,7 +271,7 @@
     <t xml:space="preserve">X_ltcg_V1 = X_ltcg_gross</t>
   </si>
   <si>
-    <t xml:space="preserve">Publishable default: K0 is built from the on-1040 realized base, so the baseline realization rate is already implicit in X.</t>
+    <t xml:space="preserve">Publishable default: Y0^K is built from the on-1040 realized base, so the baseline realization rate is already implicit in X.</t>
   </si>
   <si>
     <t xml:space="preserve">block</t>
@@ -370,7 +370,7 @@
     <t xml:space="preserve">Karger 2026 (NBER w35046) Table 39, Total column, 2025.</t>
   </si>
   <si>
-    <t xml:space="preserve">shock.variants.S.s1</t>
+    <t xml:space="preserve">shock.variants.S.theta1_k</t>
   </si>
   <si>
     <t xml:space="preserve">0.45</t>
@@ -388,7 +388,7 @@
     <t xml:space="preserve">Karger 2026 (NBER w35046) Table 19, Slow scenario, median 2030 annualized GDP growth rate.</t>
   </si>
   <si>
-    <t xml:space="preserve">shock.variants.M.s1</t>
+    <t xml:space="preserve">shock.variants.M.theta1_k</t>
   </si>
   <si>
     <t xml:space="preserve">0.462</t>
@@ -406,7 +406,7 @@
     <t xml:space="preserve">Karger 2026 (NBER w35046) Table 19, Moderate scenario, median 2030 annualized GDP growth rate.</t>
   </si>
   <si>
-    <t xml:space="preserve">shock.variants.R.s1</t>
+    <t xml:space="preserve">shock.variants.R.theta1_k</t>
   </si>
   <si>
     <t xml:space="preserve">0.487</t>
@@ -505,34 +505,34 @@
     <t xml:space="preserve">TCJA federal C-corp rate (IRC §11).</t>
   </si>
   <si>
-    <t xml:space="preserve">s1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">alpha</t>
+    <t xml:space="preserve">theta1_k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g_y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g_k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g_l</t>
   </si>
   <si>
     <t xml:space="preserve">k_inequality</t>
   </si>
   <si>
-    <t xml:space="preserve">sigma_S2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sigma_S3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L0_dollar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K0_dollar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Y0_dollar</t>
+    <t xml:space="preserve">lambda_S2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lambda_S3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">y0_l_dollar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">y0_k_dollar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">y0_dollar</t>
   </si>
   <si>
     <t xml:space="preserve">X</t>
@@ -601,7 +601,7 @@
     <t xml:space="preserve">1.0</t>
   </si>
   <si>
-    <t xml:space="preserve">Multiplier on the AI growth bump gy that sets the size of the dispersion shift in the log-affine map. Same value across all variants in a run; per-variant sigma values differ because gy differs.</t>
+    <t xml:space="preserve">Multiplier on the AI growth bump g_y that sets the size of the dispersion shift in the log-affine map. Same value across all variants in a run; per-variant lambda values differ because g_y differs.</t>
   </si>
   <si>
     <t xml:space="preserve">scenario_params.yaml: labor_inequality.k (default 1).</t>
@@ -610,40 +610,40 @@
     <t xml:space="preserve">Compressive slope (S2)</t>
   </si>
   <si>
-    <t xml:space="preserve">sigma_S2 = 1 - k_inequality * gy</t>
+    <t xml:space="preserve">lambda_S2 = 1 - k_inequality * g_y</t>
   </si>
   <si>
     <t xml:space="preserve">S: 0.949 | M: 0.933 | R: 0.896  (at k=1)</t>
   </si>
   <si>
-    <t xml:space="preserve">Compressive map: top of the ln(YiL) distribution is pulled toward the mean by (1 - sigma_S2). Rationale: AI commoditizes high-skill premia. Larger gy =&gt; more compression.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Computed in 03_shock_labor.R; gy from the macro step (per-variant). See parameters sheet.</t>
+    <t xml:space="preserve">Compressive map: top of the ln(y_l) distribution is pulled toward the mean by (1 - lambda_S2). Rationale: AI commoditizes high-skill premia. Larger g_y =&gt; more compression.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Computed in 03_shock_labor.R; g_y from the macro step (per-variant). See parameters sheet.</t>
   </si>
   <si>
     <t xml:space="preserve">Expansive slope (S3)</t>
   </si>
   <si>
-    <t xml:space="preserve">sigma_S3 = 1 + k_inequality * gy</t>
+    <t xml:space="preserve">lambda_S3 = 1 + k_inequality * g_y</t>
   </si>
   <si>
     <t xml:space="preserve">S: 1.051 | M: 1.067 | R: 1.104  (at k=1)</t>
   </si>
   <si>
-    <t xml:space="preserve">Expansive map: top of the ln(YiL) distribution is stretched away from the mean by (sigma_S3 - 1). Rationale: AI super-charges top earners (winner-take-most). Larger gy =&gt; more expansion.</t>
+    <t xml:space="preserve">Expansive map: top of the ln(y_l) distribution is stretched away from the mean by (lambda_S3 - 1). Rationale: AI super-charges top earners (winner-take-most). Larger g_y =&gt; more expansion.</t>
   </si>
   <si>
     <t xml:space="preserve">Aggregate anchor</t>
   </si>
   <si>
-    <t xml:space="preserve">mu1 via uniroot s.t. sum(weight * exp(mu1 + sigma * (ln(YiL0) - mu0))) = L1$</t>
+    <t xml:space="preserve">mu1 via uniroot s.t. sum(weight * exp(mu1 + lambda * (ln(y_l) - mu0))) = Y1^L$</t>
   </si>
   <si>
     <t xml:space="preserve">varies by cell</t>
   </si>
   <si>
-    <t xml:space="preserve">Intercept mu1 is solved to preserve the aggregate labor income target L1$ from the macro step. mu0 is the weighted mean of ln(YiL) on positive-labor units in the baseline.</t>
+    <t xml:space="preserve">Intercept mu1 is solved to preserve the aggregate labor income target Y1^L$ from the macro step. mu0 is the weighted mean of ln(y_l) on positive-labor units in the baseline.</t>
   </si>
   <si>
     <t xml:space="preserve">Computed in 03_shock_labor.R.</t>
@@ -688,13 +688,13 @@
     <t xml:space="preserve">Calibrated corporate-base scale factor</t>
   </si>
   <si>
-    <t xml:space="preserve">eta = tau_stat * (K0$ * kappa_corp) / CBO_CIT$</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calibrated at runtime from K0$</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calibrated at runtime by compute_macro_targets() so that tau_stat * (K0$ * kappa_corp) / eta matches CBO_CIT$ at baseline. eta absorbs household-realized-vs-pre-realization wedge plus statutory-vs-effective gap.</t>
+    <t xml:space="preserve">eta = tau_stat * (Y0^K$ * kappa_corp) / CBO_CIT$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calibrated at runtime from Y0^K$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calibrated at runtime by compute_macro_targets() so that tau_stat * (Y0^K$ * kappa_corp) / eta matches CBO_CIT$ at baseline. eta absorbs household-realized-vs-pre-realization wedge plus statutory-vs-effective gap.</t>
   </si>
   <si>
     <t xml:space="preserve">Derived in 04_allocate_capital.R::compute_macro_targets. See parameters sheet.</t>
@@ -703,7 +703,7 @@
     <t xml:space="preserve">Capital flow (gross)</t>
   </si>
   <si>
-    <t xml:space="preserve">X = K0$ * gk</t>
+    <t xml:space="preserve">X = Y0^K$ * g_k</t>
   </si>
   <si>
     <t xml:space="preserve">varies by variant</t>
@@ -733,7 +733,7 @@
     <t xml:space="preserve">Macro CIT delta</t>
   </si>
   <si>
-    <t xml:space="preserve">delta_R_CIT = tau_stat * kappa_corp * X / eta ≡ X * CBO_CIT$ / K0$</t>
+    <t xml:space="preserve">delta_R_CIT = tau_stat * kappa_corp * X / eta ≡ X * CBO_CIT$ / Y0^K$</t>
   </si>
   <si>
     <t xml:space="preserve">varies by variant only</t>
@@ -1051,40 +1051,40 @@
     <t xml:space="preserve">Shock variant: S (Slow), M (Moderate), R (Rapid). Karger 2026 NBER w35046, Tables 19 / 39.</t>
   </si>
   <si>
-    <t xml:space="preserve">Factor-share mode. R = reallocate (Karger s1 from yaml). F = fixed (s1 := 1 - L0 so the labor-capital split is preserved). Same gy under both modes; F has gk = gy and alpha = 1 by construction.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Period-1 capital share target = 1 - period-1 labor share.</t>
+    <t xml:space="preserve">Factor-share mode. R = reallocate (Karger theta1_k from yaml). F = fixed (theta1_k := theta0_k so the labor-capital split is preserved). Same g_y under both modes; F has g_k = g_l = g_y by construction.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Post-shock capital share target = 1 - post-shock labor share.</t>
   </si>
   <si>
     <t xml:space="preserve">Multiplicative AI bump on the no-AI baseline-year level: (1 + r_ai_annual)^horizon / cum_base - 1, where r_ai_annual is Karger Table 19 median GDP CAGR under AI and cum_base = (1 + g_2026) * (1 + g_2027plus)^(horizon-1) is the CBO baseline path (publication 62105). Horizon = baseline_year - 2025 (= 5 for 2030).</t>
   </si>
   <si>
-    <t xml:space="preserve">Capital factor growth rate over the horizon; derived in 02_params.R from (s1, gy, L0).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Labor growth as a multiple of capital growth; labor grows at alpha * gk.</t>
+    <t xml:space="preserve">Cumulative capital-income growth rate over the horizon; derived in 02_params.R from (theta1_k, g_y, theta0_l).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cumulative labor-income growth rate over the horizon. Labor grows at g_l (equals g_k under fixed share; below g_k under reallocate).</t>
   </si>
   <si>
     <t xml:space="preserve">Multiplier on g_y that sets the S2/S3 dispersion shift. From config: labor_inequality.k. Same value across all variants in a run.</t>
   </si>
   <si>
-    <t xml:space="preserve">S2 (compressive) log-affine slope = 1 - k_inequality * gy. Per-variant since gy varies.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S3 (expansive) log-affine slope = 1 + k_inequality * gy. Per-variant since gy varies.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Microsim baseline aggregate labor income, sum(weight*YiL) in $.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Microsim baseline aggregate capital income, sum(weight*YiK) in $.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L0_dollar + K0_dollar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Implied capital flow = K0_dollar * gk ($).</t>
+    <t xml:space="preserve">S2 (compressive) log-affine slope = 1 - k_inequality * g_y. Per-variant since g_y varies.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S3 (expansive) log-affine slope = 1 + k_inequality * g_y. Per-variant since g_y varies.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Microsim baseline aggregate labor income, sum(weight*y_l) in $.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Microsim baseline aggregate capital income, sum(weight*y_k) in $.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">y0_l_dollar + y0_k_dollar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implied capital flow = y0_k_dollar * g_k ($).</t>
   </si>
   <si>
     <t xml:space="preserve">X reaches households in full: CIT is modeled upstream of household realizations, so X_to_units = X ($).</t>
@@ -1099,10 +1099,10 @@
     <t xml:space="preserve">CBO baseline-year CIT revenue level ($). cit_to_gdp_baseline_year * gdp_baseline_year_B * 1e9. Anchors the eta calibration.</t>
   </si>
   <si>
-    <t xml:space="preserve">Calibrated corporate-base scale factor (eta_corp). cit_statutory * (K0_dollar * kappa_corp) / cbo_cit_baseline_dollar. Absorbs both household-realized-vs-pre-realization wedge and the statutory-vs-effective gap.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Off-microsim CIT revenue change ($). cit_statutory * kappa_corp * X / eta_corp; algebraically equals X * cbo_cit_baseline_dollar / K0_dollar. Add to microsim total in 09_tables_figures.R.</t>
+    <t xml:space="preserve">Calibrated corporate-base scale factor (eta_corp). cit_statutory * (y0_k_dollar * kappa_corp) / cbo_cit_baseline_dollar. Absorbs both household-realized-vs-pre-realization wedge and the statutory-vs-effective gap.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Off-microsim CIT revenue change ($). cit_statutory * kappa_corp * X / eta_corp; algebraically equals X * cbo_cit_baseline_dollar / y0_k_dollar. Add to microsim total in 09_tables_figures.R.</t>
   </si>
   <si>
     <t xml:space="preserve">Capital flow X_to_units allocated to qualified dividends ($B). 30% of public-equity allocation (per config/asset_to_income_map.csv).</t>
@@ -1297,49 +1297,64 @@
     <t xml:space="preserve">top_5_pct</t>
   </si>
   <si>
-    <t xml:space="preserve">variant_label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">share_mode_label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">labor_label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">r_ai_annual_target</t>
-  </si>
-  <si>
-    <t xml:space="preserve">delta_rev_to_gdp_cbo_pp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prod_bump_pp_per_yr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blsmm_gstar_year_pct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blsmm_annualized_growth_horizon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blsmm_year_real_growth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blsmm_rgfr_year_pct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blsmm_rgfop_year_pct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blsmm_debt_year_B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blsmm_gdp_nominal_year_B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blsmm_debt_to_gdp_year_pct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">delta_debt_to_gdp_vs_baseline_pp</t>
+    <t xml:space="preserve">Scenario ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI Adoption</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share Mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share Mode (label)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Labor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Labor Scenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Realization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI GDP CAGR Target</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Δ Revenue-to-GDP vs CBO (pp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Productivity Bump (pp/yr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GDP Growth g* (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annualized Growth (2025–Year)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real GDP Growth (Year)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Federal Revenue Path rgfr* (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rgfop* (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Debt ($B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nominal GDP ($B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Debt-to-GDP (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Δ Debt-to-GDP vs Baseline (pp)</t>
   </si>
   <si>
     <t xml:space="preserve">blsmm_baseline</t>
@@ -20122,69 +20137,69 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>303</v>
+        <v>423</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>424</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>45</v>
+        <v>426</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>57</v>
+        <v>428</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>76</v>
+        <v>430</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>426</v>
+        <v>431</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>430</v>
+        <v>435</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>431</v>
+        <v>436</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>432</v>
+        <v>437</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>434</v>
+        <v>439</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>435</v>
+        <v>440</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>436</v>
+        <v>441</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>437</v>
+        <v>442</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>438</v>
+        <v>443</v>
       </c>
       <c r="B2"/>
       <c r="C2"/>
@@ -22016,7 +22031,7 @@
   <cols>
     <col min="1" max="1" width="7.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="10.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="5.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="8.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="11.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="11.71" hidden="0" customWidth="1"/>
@@ -22147,7 +22162,7 @@
         <v>0.0172117163991912</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.183182342457595</v>
+        <v>-0.00315288252771963</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
@@ -22233,7 +22248,7 @@
         <v>0.0754166612691227</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0545829695654936</v>
+        <v>0.00411646532678367</v>
       </c>
       <c r="G3" t="n">
         <v>1</v>
@@ -22319,7 +22334,7 @@
         <v>0.172812402611785</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.0545835382921483</v>
+        <v>-0.00943271239531852</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
@@ -22405,7 +22420,7 @@
         <v>0.00590936399475563</v>
       </c>
       <c r="F5" t="n">
-        <v>1.00000000000001</v>
+        <v>0.0059093639947557</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
@@ -22491,7 +22506,7 @@
         <v>0.0358450525211244</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0.0358450525211244</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>
@@ -22577,7 +22592,7 @@
         <v>0.0716663637828425</v>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>0.0716663637828425</v>
       </c>
       <c r="G7" t="n">
         <v>1</v>
@@ -22658,7 +22673,7 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="22.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="76.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="78.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="40.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="60.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="60.71" hidden="0" customWidth="1"/>

</xml_diff>

<commit_message>
results: regenerate 2030 deliverables (vintage 202607091035)
Full 18-cell grid re-run; xlsx bundles + figure suite refreshed,
including BLSMM debt/GDP sheets and figures. Tax-Simulator output
written to the production root.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/aggregates/ai_fiscal_2030_latest.xlsx
+++ b/results/aggregates/ai_fiscal_2030_latest.xlsx
@@ -37,7 +37,7 @@
     <t xml:space="preserve">Generated</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-06-30 00:20:45 EDT</t>
+    <t xml:space="preserve">2026-07-09 10:40:54 EDT</t>
   </si>
   <si>
     <t xml:space="preserve">Policy year</t>
@@ -49,13 +49,13 @@
     <t xml:space="preserve">Tax-Simulator vintage</t>
   </si>
   <si>
-    <t xml:space="preserve">202606300013</t>
+    <t xml:space="preserve">202607091035</t>
   </si>
   <si>
     <t xml:space="preserve">Tax-Simulator output root</t>
   </si>
   <si>
-    <t xml:space="preserve">/nfs/roberts/scratch/pi_nrs36/ji252/model_data/Tax-Simulator/v1/202606300013</t>
+    <t xml:space="preserve">/nfs/roberts/project/pi_nrs36/shared/model_data/Tax-Simulator/v1/202607091035</t>
   </si>
   <si>
     <t xml:space="preserve">Runscript</t>
@@ -85,13 +85,13 @@
     <t xml:space="preserve">AI-Fiscal git rev</t>
   </si>
   <si>
-    <t xml:space="preserve">4a1111ae1e12</t>
+    <t xml:space="preserve">74de5986e5ff</t>
   </si>
   <si>
     <t xml:space="preserve">Orchestrator argv</t>
   </si>
   <si>
-    <t xml:space="preserve">--overwrite --multicore scenario</t>
+    <t xml:space="preserve">--multicore scenario --overwrite</t>
   </si>
   <si>
     <t xml:space="preserve">axis</t>
@@ -319,7 +319,7 @@
     <t xml:space="preserve">sourced</t>
   </si>
   <si>
-    <t xml:space="preserve">CBO 2025 Budget and Economic Outlook (publication 62105), Table 1, real GDP growth for 2026.</t>
+    <t xml:space="preserve">CBO February 2026 Budget and Economic Outlook: 2026 to 2036 (publication 62105), Table 1, real GDP growth for 2026.</t>
   </si>
   <si>
     <t xml:space="preserve">cbo_baseline.g_2027plus</t>
@@ -328,7 +328,7 @@
     <t xml:space="preserve">0.018</t>
   </si>
   <si>
-    <t xml:space="preserve">CBO 2025 Budget and Economic Outlook (publication 62105), Table 1, real GDP growth for 2027 and onward (held flat at 1.8%/yr).</t>
+    <t xml:space="preserve">CBO February 2026 Budget and Economic Outlook: 2026 to 2036 (publication 62105), Table 1, real GDP growth for 2027 and onward (held flat at 1.8%/yr).</t>
   </si>
   <si>
     <t xml:space="preserve">cbo_baseline.gdp_baseline_year_B</t>
@@ -337,7 +337,7 @@
     <t xml:space="preserve">37391</t>
   </si>
   <si>
-    <t xml:space="preserve">CBO 2025 Budget and Economic Outlook (publication 62105), 2030 nominal GDP.</t>
+    <t xml:space="preserve">CBO February 2026 Budget and Economic Outlook: 2026 to 2036 (publication 62105), 2030 nominal GDP.</t>
   </si>
   <si>
     <t xml:space="preserve">cbo_baseline.rev_to_gdp_baseline_year</t>
@@ -346,7 +346,7 @@
     <t xml:space="preserve">0.177</t>
   </si>
   <si>
-    <t xml:space="preserve">CBO 2025 Budget and Economic Outlook (publication 62105), Table 1, 2030 total federal revenue as a share of GDP.</t>
+    <t xml:space="preserve">CBO February 2026 Budget and Economic Outlook: 2026 to 2036 (publication 62105), Table 1, 2030 total federal revenue as a share of GDP.</t>
   </si>
   <si>
     <t xml:space="preserve">cbo_baseline.cit_to_gdp_baseline_year</t>
@@ -355,7 +355,7 @@
     <t xml:space="preserve">0.013</t>
   </si>
   <si>
-    <t xml:space="preserve">CBO 2025 Budget and Economic Outlook (publication 62105), Table 1, 2030 federal corporate-tax revenue as a share of GDP.</t>
+    <t xml:space="preserve">CBO February 2026 Budget and Economic Outlook: 2026 to 2036 (publication 62105), Table 1, 2030 federal corporate-tax revenue as a share of GDP.</t>
   </si>
   <si>
     <t xml:space="preserve">shock</t>
@@ -448,7 +448,7 @@
     <t xml:space="preserve">99.99</t>
   </si>
   <si>
-    <t xml:space="preserve">Smith-Yagan-Zidar 2019 active-profit split, tax-unit-level threshold.</t>
+    <t xml:space="preserve">Saez and Zucman (2020) active-profit split, tax-unit-level threshold.</t>
   </si>
   <si>
     <t xml:space="preserve">passthrough.wage_threshold_conditioning</t>
@@ -457,7 +457,7 @@
     <t xml:space="preserve">positive_wages</t>
   </si>
   <si>
-    <t xml:space="preserve">'positive_wages' matches the W-2 universe per SYZ.</t>
+    <t xml:space="preserve">'positive_wages' matches the W-2 universe per SZ.</t>
   </si>
   <si>
     <t xml:space="preserve">passthrough.active_below_capital_share</t>
@@ -466,7 +466,7 @@
     <t xml:space="preserve">0.25</t>
   </si>
   <si>
-    <t xml:space="preserve">Smith-Yagan-Zidar 2019: 25% of below-W* active profit -&gt; capital.</t>
+    <t xml:space="preserve">Saez and Zucman (2020): 25% of below-W* active profit -&gt; capital.</t>
   </si>
   <si>
     <t xml:space="preserve">passthrough.active_above_capital_share</t>
@@ -475,13 +475,13 @@
     <t xml:space="preserve">0.75</t>
   </si>
   <si>
-    <t xml:space="preserve">Smith-Yagan-Zidar 2019: 75% of above-W* active profit -&gt; capital.</t>
+    <t xml:space="preserve">Saez and Zucman (2020): 75% of above-W* active profit -&gt; capital.</t>
   </si>
   <si>
     <t xml:space="preserve">passthrough.passive_capital_share</t>
   </si>
   <si>
-    <t xml:space="preserve">Smith-Yagan-Zidar 2019: 75% of passive profit -&gt; capital.</t>
+    <t xml:space="preserve">Saez and Zucman (2020): 75% of passive profit -&gt; capital.</t>
   </si>
   <si>
     <t xml:space="preserve">corporate</t>
@@ -664,7 +664,7 @@
     <t xml:space="preserve">0.50 (narrow definition)</t>
   </si>
   <si>
-    <t xml:space="preserve">Narrow definition. S-corp + partnership profits are routed separately to households via the Smith-Yagan-Zidar 2019 split in 01_load_data.R, so they're already in the IIT side. Inclusive definition (S-corp counted) gives 0.62. Sensitivity range [0.45, 0.65].</t>
+    <t xml:space="preserve">Narrow definition. S-corp + partnership profits are routed separately to households via the Saez and Zucman (2020) split in 01_load_data.R, so they're already in the IIT side. Inclusive definition (S-corp counted) gives 0.62. Sensitivity range [0.45, 0.65].</t>
   </si>
   <si>
     <t xml:space="preserve">scenario_params.yaml: corporate.kappa_corp; NIPA 2024 Z.1 F.3.</t>
@@ -679,7 +679,7 @@
     <t xml:space="preserve">cit_to_gdp_baseline_year * gdp_baseline_year_B$ (from scenario_params.yaml)</t>
   </si>
   <si>
-    <t xml:space="preserve">CBO 2025 Budget and Economic Outlook (publication 62105), Table 1, 2030 federal CIT / GDP, applied to 2030 nominal GDP.</t>
+    <t xml:space="preserve">CBO February 2026 Budget and Economic Outlook: 2026 to 2036 (publication 62105), Table 1, 2030 federal CIT / GDP, applied to 2030 nominal GDP.</t>
   </si>
   <si>
     <t xml:space="preserve">scenario_params.yaml: cbo_baseline.cit_to_gdp_baseline_year × gdp_baseline_year_B.</t>
@@ -829,10 +829,10 @@
     <t xml:space="preserve">proprietors_capital_share</t>
   </si>
   <si>
-    <t xml:space="preserve">Smith-Yagan-Zidar 2019 (passthrough split)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Symmetric SYZ rule averages to ~50% capital across the population</t>
+    <t xml:space="preserve">Saez and Zucman (2020) (passthrough split)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Symmetric SZ rule averages to ~50% capital across the population</t>
   </si>
   <si>
     <t xml:space="preserve">scorp_share_of_BEA_corporate_profits</t>

</xml_diff>